<commit_message>
Update vault (2026-08-11 23:17 IST)
</commit_message>
<xml_diff>
--- a/sem_3/assignments/SDA/CustomerCleanup_Chayan_Lab4.xlsx
+++ b/sem_3/assignments/SDA/CustomerCleanup_Chayan_Lab4.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chaya\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Aditya\mainframe\vault\sem_3\assignments\SDA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{621FBEA1-A72F-430B-B352-CCCBB765A4DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92AB8DAD-C927-480B-A33F-D9D82ACBE256}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8460" yWindow="0" windowWidth="14676" windowHeight="12336" activeTab="1" xr2:uid="{32266424-75D2-420C-98EF-05F339009423}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{32266424-75D2-420C-98EF-05F339009423}"/>
   </bookViews>
   <sheets>
     <sheet name="customer_data" sheetId="2" r:id="rId1"/>
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="222" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="144">
   <si>
     <t>Customer ID</t>
   </si>
@@ -104,9 +104,6 @@
     <t>diya.rao1@example.com</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
     <t>Jaipur</t>
   </si>
   <si>
@@ -419,9 +416,6 @@
     <t>CUST0034</t>
   </si>
   <si>
-    <t xml:space="preserve">Anika Gupta </t>
-  </si>
-  <si>
     <t>anika.gupta12@example.com</t>
   </si>
   <si>
@@ -483,6 +477,9 @@
   </si>
   <si>
     <t xml:space="preserve"> Ahmedabad</t>
+  </si>
+  <si>
+    <t>Anika Gupta</t>
   </si>
 </sst>
 </file>
@@ -970,17 +967,13 @@
     <xf numFmtId="0" fontId="2" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1028,12 +1021,6 @@
   </cellStyles>
   <dxfs count="11">
     <dxf>
-      <numFmt numFmtId="165" formatCode="&quot;₹&quot;\ #,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
@@ -1043,6 +1030,9 @@
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="165" formatCode="&quot;₹&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="164" formatCode="dd/mmm/yyyy"/>
     </dxf>
     <dxf>
@@ -1050,6 +1040,9 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
@@ -1103,16 +1096,16 @@
     <tableColumn id="1" xr3:uid="{85EDDAFB-81CC-4989-ADA4-A83A853EE229}" uniqueName="1" name="Customer ID" queryTableFieldId="1" dataDxfId="10"/>
     <tableColumn id="2" xr3:uid="{779D19FC-5F19-4420-BE29-4D36DA1A9331}" uniqueName="2" name="Full Name" queryTableFieldId="2" dataDxfId="9"/>
     <tableColumn id="3" xr3:uid="{EB10A194-3451-4191-B3DC-105765CC5537}" uniqueName="3" name="Email" queryTableFieldId="3" dataDxfId="8"/>
-    <tableColumn id="4" xr3:uid="{BA0648A9-992E-4115-9FCD-44F64298529C}" uniqueName="4" name="Phone" queryTableFieldId="4" dataDxfId="1"/>
-    <tableColumn id="5" xr3:uid="{0B09E690-2AC2-4B93-B5C6-C5058F959385}" uniqueName="5" name="City" queryTableFieldId="5" dataDxfId="7"/>
-    <tableColumn id="6" xr3:uid="{F3E7DEB6-898F-4CBF-9074-EF4239484655}" uniqueName="6" name="State" queryTableFieldId="6" dataDxfId="6"/>
-    <tableColumn id="7" xr3:uid="{75042A5B-1E95-4FA4-970F-3591FCAEB821}" uniqueName="7" name="Signup Date" queryTableFieldId="7" dataDxfId="5"/>
-    <tableColumn id="8" xr3:uid="{E5F88D94-D9A5-49F9-8B1E-C00F359BC29E}" uniqueName="8" name="Total Purchases" queryTableFieldId="8" dataDxfId="0"/>
-    <tableColumn id="9" xr3:uid="{9D9FA1BF-1A74-42C6-B7F2-61274BD0DAA6}" uniqueName="9" name="Membership Tier" queryTableFieldId="9" dataDxfId="4"/>
-    <tableColumn id="10" xr3:uid="{6B2A2734-5BA5-4CEB-83CD-C3244FB2094F}" uniqueName="10" name="Review ?" queryTableFieldId="10" dataDxfId="3">
+    <tableColumn id="4" xr3:uid="{BA0648A9-992E-4115-9FCD-44F64298529C}" uniqueName="4" name="Phone" queryTableFieldId="4" dataDxfId="7"/>
+    <tableColumn id="5" xr3:uid="{0B09E690-2AC2-4B93-B5C6-C5058F959385}" uniqueName="5" name="City" queryTableFieldId="5" dataDxfId="6"/>
+    <tableColumn id="6" xr3:uid="{F3E7DEB6-898F-4CBF-9074-EF4239484655}" uniqueName="6" name="State" queryTableFieldId="6" dataDxfId="5"/>
+    <tableColumn id="7" xr3:uid="{75042A5B-1E95-4FA4-970F-3591FCAEB821}" uniqueName="7" name="Signup Date" queryTableFieldId="7" dataDxfId="4"/>
+    <tableColumn id="8" xr3:uid="{E5F88D94-D9A5-49F9-8B1E-C00F359BC29E}" uniqueName="8" name="Total Purchases" queryTableFieldId="8" dataDxfId="3"/>
+    <tableColumn id="9" xr3:uid="{9D9FA1BF-1A74-42C6-B7F2-61274BD0DAA6}" uniqueName="9" name="Membership Tier" queryTableFieldId="9" dataDxfId="2"/>
+    <tableColumn id="10" xr3:uid="{6B2A2734-5BA5-4CEB-83CD-C3244FB2094F}" uniqueName="10" name="Review ?" queryTableFieldId="10" dataDxfId="1">
       <calculatedColumnFormula>IF(OR(M2&gt;1,O2&gt;1),"Review","OK")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{93EB9993-D7E9-40E1-9722-83DD82B06825}" uniqueName="11" name="City(Cleaned" queryTableFieldId="11" dataDxfId="2">
+    <tableColumn id="11" xr3:uid="{93EB9993-D7E9-40E1-9722-83DD82B06825}" uniqueName="11" name="City(Cleaned" queryTableFieldId="11" dataDxfId="0">
       <calculatedColumnFormula>PROPER(TRIM(customer_data[[#This Row],[City]]))</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1418,25 +1411,25 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B3871D7-D974-4A74-9751-D43AEF05518B}">
   <dimension ref="A1:O35"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="32.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.33203125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="32.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.28515625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="12.140625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="12" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.88671875" style="3" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="17.109375" style="5" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="18.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17.140625" style="5" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18.7109375" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="12" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="32.6640625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="18.44140625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="18.6640625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="18.109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="32.7109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="18.42578125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="18.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1483,7 +1476,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>15</v>
       </c>
@@ -1494,13 +1487,13 @@
         <v>17</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="E2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F2" t="s">
         <v>19</v>
-      </c>
-      <c r="F2" t="s">
-        <v>20</v>
       </c>
       <c r="G2" s="3">
         <v>45544</v>
@@ -1509,7 +1502,7 @@
         <v>18267</v>
       </c>
       <c r="I2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="J2" t="str">
         <f t="shared" ref="J2:J31" si="0">IF(OR(M2&gt;1,O2&gt;1),"Review","OK")</f>
@@ -1524,7 +1517,7 @@
         <v>diya.rao1@example.com</v>
       </c>
       <c r="M2">
-        <f>COUNTIF($C$2:$C$31,L2)</f>
+        <f t="shared" ref="M2:M31" si="1">COUNTIF($C$2:$C$31,L2)</f>
         <v>1</v>
       </c>
       <c r="N2" t="str">
@@ -1532,28 +1525,28 @@
         <v>Diya Rao</v>
       </c>
       <c r="O2">
-        <f>COUNTIF($B$2:$B$31,N2)</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
+        <f t="shared" ref="O2:O31" si="2">COUNTIF($B$2:$B$31,N2)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B3" t="s">
         <v>22</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C3" t="s">
         <v>23</v>
-      </c>
-      <c r="C3" t="s">
-        <v>24</v>
       </c>
       <c r="D3" s="1">
         <v>9177981348</v>
       </c>
       <c r="E3" t="s">
+        <v>24</v>
+      </c>
+      <c r="F3" t="s">
         <v>25</v>
-      </c>
-      <c r="F3" t="s">
-        <v>26</v>
       </c>
       <c r="G3" s="3">
         <v>45602</v>
@@ -1562,7 +1555,7 @@
         <v>31080</v>
       </c>
       <c r="I3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="J3" t="str">
         <f t="shared" si="0"/>
@@ -1577,7 +1570,7 @@
         <v>ananya.bhatt2@example.com</v>
       </c>
       <c r="M3">
-        <f>COUNTIF($C$2:$C$31,L3)</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="N3" t="str">
@@ -1585,28 +1578,28 @@
         <v>Ananya Bhatt</v>
       </c>
       <c r="O3">
-        <f>COUNTIF($B$2:$B$31,N3)</f>
+        <f t="shared" si="2"/>
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B4" t="s">
         <v>28</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
         <v>29</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="E4" t="s">
         <v>31</v>
       </c>
-      <c r="E4" t="s">
+      <c r="F4" t="s">
         <v>32</v>
-      </c>
-      <c r="F4" t="s">
-        <v>33</v>
       </c>
       <c r="G4" s="3">
         <v>45520</v>
@@ -1615,7 +1608,7 @@
         <v>21186</v>
       </c>
       <c r="I4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="J4" t="str">
         <f t="shared" si="0"/>
@@ -1630,7 +1623,7 @@
         <v>arjun.chauhan3@example.com</v>
       </c>
       <c r="M4">
-        <f>COUNTIF($C$2:$C$31,L4)</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="N4" t="str">
@@ -1638,28 +1631,28 @@
         <v>Arjun Chauhan</v>
       </c>
       <c r="O4">
-        <f>COUNTIF($B$2:$B$31,N4)</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>33</v>
+      </c>
+      <c r="B5" t="s">
         <v>34</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C5" t="s">
         <v>35</v>
-      </c>
-      <c r="C5" t="s">
-        <v>36</v>
       </c>
       <c r="D5" s="1">
         <v>9487266582</v>
       </c>
       <c r="E5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F5" t="s">
         <v>19</v>
-      </c>
-      <c r="F5" t="s">
-        <v>20</v>
       </c>
       <c r="G5" s="3">
         <v>45445</v>
@@ -1668,7 +1661,7 @@
         <v>11054</v>
       </c>
       <c r="I5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="J5" t="str">
         <f t="shared" si="0"/>
@@ -1683,7 +1676,7 @@
         <v>isha.reddy4@example.com</v>
       </c>
       <c r="M5">
-        <f>COUNTIF($C$2:$C$31,L5)</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="N5" t="str">
@@ -1691,28 +1684,28 @@
         <v>Isha Reddy</v>
       </c>
       <c r="O5">
-        <f>COUNTIF($B$2:$B$31,N5)</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>36</v>
+      </c>
+      <c r="B6" t="s">
         <v>37</v>
       </c>
-      <c r="B6" t="s">
+      <c r="C6" t="s">
         <v>38</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D6" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="E6" t="s">
         <v>39</v>
       </c>
-      <c r="D6" s="1" t="s">
-        <v>130</v>
-      </c>
-      <c r="E6" t="s">
+      <c r="F6" t="s">
         <v>40</v>
-      </c>
-      <c r="F6" t="s">
-        <v>41</v>
       </c>
       <c r="G6" s="3">
         <v>45417</v>
@@ -1721,7 +1714,7 @@
         <v>39482</v>
       </c>
       <c r="I6" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="J6" t="str">
         <f t="shared" si="0"/>
@@ -1736,7 +1729,7 @@
         <v>ishaan.sharma5@example.com</v>
       </c>
       <c r="M6">
-        <f>COUNTIF($C$2:$C$31,L6)</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="N6" t="str">
@@ -1744,28 +1737,28 @@
         <v>Ishaan Sharma</v>
       </c>
       <c r="O6">
-        <f>COUNTIF($B$2:$B$31,N6)</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>41</v>
+      </c>
+      <c r="B7" t="s">
         <v>42</v>
       </c>
-      <c r="B7" t="s">
+      <c r="C7" t="s">
         <v>43</v>
-      </c>
-      <c r="C7" t="s">
-        <v>44</v>
       </c>
       <c r="D7" s="1">
         <v>9394263945</v>
       </c>
       <c r="E7" t="s">
+        <v>44</v>
+      </c>
+      <c r="F7" t="s">
         <v>45</v>
-      </c>
-      <c r="F7" t="s">
-        <v>46</v>
       </c>
       <c r="G7" s="3">
         <v>46166</v>
@@ -1774,7 +1767,7 @@
         <v>25526</v>
       </c>
       <c r="I7" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="J7" t="str">
         <f t="shared" si="0"/>
@@ -1789,7 +1782,7 @@
         <v>aarav.verma6@example.com</v>
       </c>
       <c r="M7">
-        <f>COUNTIF($C$2:$C$31,L7)</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="N7" t="str">
@@ -1797,28 +1790,28 @@
         <v>Aarav Verma</v>
       </c>
       <c r="O7">
-        <f>COUNTIF($B$2:$B$31,N7)</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>46</v>
+      </c>
+      <c r="B8" t="s">
         <v>47</v>
       </c>
-      <c r="B8" t="s">
+      <c r="C8" t="s">
         <v>48</v>
-      </c>
-      <c r="C8" t="s">
-        <v>49</v>
       </c>
       <c r="D8" s="1">
         <v>9752331677</v>
       </c>
       <c r="E8" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="F8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G8" s="3">
         <v>46185</v>
@@ -1827,7 +1820,7 @@
         <v>42499</v>
       </c>
       <c r="I8" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="J8" t="str">
         <f t="shared" si="0"/>
@@ -1842,7 +1835,7 @@
         <v>aditya.das7@example.com</v>
       </c>
       <c r="M8">
-        <f>COUNTIF($C$2:$C$31,L8)</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="N8" t="str">
@@ -1850,28 +1843,28 @@
         <v>Aditya Das</v>
       </c>
       <c r="O8">
-        <f>COUNTIF($B$2:$B$31,N8)</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>50</v>
+      </c>
+      <c r="B9" t="s">
         <v>51</v>
       </c>
-      <c r="B9" t="s">
+      <c r="C9" t="s">
         <v>52</v>
       </c>
-      <c r="C9" t="s">
+      <c r="D9" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="D9" s="1" t="s">
+      <c r="E9" t="s">
         <v>54</v>
       </c>
-      <c r="E9" t="s">
+      <c r="F9" t="s">
         <v>55</v>
-      </c>
-      <c r="F9" t="s">
-        <v>56</v>
       </c>
       <c r="G9" s="3">
         <v>45477</v>
@@ -1880,7 +1873,7 @@
         <v>6704</v>
       </c>
       <c r="I9" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="J9" t="str">
         <f t="shared" si="0"/>
@@ -1895,7 +1888,7 @@
         <v>aditya.rao8@example.com</v>
       </c>
       <c r="M9">
-        <f>COUNTIF($C$2:$C$31,L9)</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="N9" t="str">
@@ -1903,28 +1896,28 @@
         <v>Aditya Rao</v>
       </c>
       <c r="O9">
-        <f>COUNTIF($B$2:$B$31,N9)</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>56</v>
+      </c>
+      <c r="B10" t="s">
         <v>57</v>
       </c>
-      <c r="B10" t="s">
+      <c r="C10" t="s">
         <v>58</v>
       </c>
-      <c r="C10" t="s">
-        <v>59</v>
-      </c>
       <c r="D10" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="E10" t="s">
+        <v>31</v>
+      </c>
+      <c r="F10" t="s">
         <v>32</v>
-      </c>
-      <c r="F10" t="s">
-        <v>33</v>
       </c>
       <c r="G10" s="3">
         <v>45755</v>
@@ -1933,7 +1926,7 @@
         <v>41402</v>
       </c>
       <c r="I10" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="J10" t="str">
         <f t="shared" si="0"/>
@@ -1948,7 +1941,7 @@
         <v>siddharth.kapoor9@example.com</v>
       </c>
       <c r="M10">
-        <f>COUNTIF($C$2:$C$31,L10)</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="N10" t="str">
@@ -1956,28 +1949,28 @@
         <v>Siddharth Kapoor</v>
       </c>
       <c r="O10">
-        <f>COUNTIF($B$2:$B$31,N10)</f>
+        <f t="shared" si="2"/>
         <v>2</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>60</v>
+      </c>
+      <c r="B11" t="s">
         <v>61</v>
       </c>
-      <c r="B11" t="s">
-        <v>62</v>
-      </c>
       <c r="C11" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="E11" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="F11" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G11" s="3">
         <v>45552</v>
@@ -1986,7 +1979,7 @@
         <v>7212</v>
       </c>
       <c r="I11" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="J11" t="str">
         <f t="shared" si="0"/>
@@ -2001,7 +1994,7 @@
         <v>not provided</v>
       </c>
       <c r="M11">
-        <f>COUNTIF($C$2:$C$31,L11)</f>
+        <f t="shared" si="1"/>
         <v>4</v>
       </c>
       <c r="N11" t="str">
@@ -2009,28 +2002,28 @@
         <v>Pooja Chauhan</v>
       </c>
       <c r="O11">
-        <f>COUNTIF($B$2:$B$31,N11)</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.3">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
+        <v>62</v>
+      </c>
+      <c r="B12" t="s">
         <v>63</v>
       </c>
-      <c r="B12" t="s">
-        <v>64</v>
-      </c>
       <c r="C12" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="D12" s="1">
         <v>9399178390</v>
       </c>
       <c r="E12" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F12" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="G12" s="3">
         <v>45413</v>
@@ -2039,7 +2032,7 @@
         <v>2334</v>
       </c>
       <c r="I12" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="J12" t="str">
         <f t="shared" si="0"/>
@@ -2054,7 +2047,7 @@
         <v>not provided</v>
       </c>
       <c r="M12">
-        <f>COUNTIF($C$2:$C$31,L12)</f>
+        <f t="shared" si="1"/>
         <v>4</v>
       </c>
       <c r="N12" t="str">
@@ -2062,28 +2055,28 @@
         <v>Nikhil Verma</v>
       </c>
       <c r="O12">
-        <f>COUNTIF($B$2:$B$31,N12)</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.3">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
+        <v>65</v>
+      </c>
+      <c r="B13" t="s">
         <v>66</v>
       </c>
-      <c r="B13" t="s">
+      <c r="C13" t="s">
         <v>67</v>
       </c>
-      <c r="C13" t="s">
+      <c r="D13" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="D13" s="1" t="s">
-        <v>69</v>
-      </c>
       <c r="E13" t="s">
+        <v>18</v>
+      </c>
+      <c r="F13" t="s">
         <v>19</v>
-      </c>
-      <c r="F13" t="s">
-        <v>20</v>
       </c>
       <c r="G13" s="3">
         <v>45687</v>
@@ -2092,7 +2085,7 @@
         <v>30329</v>
       </c>
       <c r="I13" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="J13" t="str">
         <f t="shared" si="0"/>
@@ -2107,7 +2100,7 @@
         <v>pooja.kapoor13@example.com</v>
       </c>
       <c r="M13">
-        <f>COUNTIF($C$2:$C$31,L13)</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="N13" t="str">
@@ -2115,28 +2108,28 @@
         <v>Pooja Kapoor</v>
       </c>
       <c r="O13">
-        <f>COUNTIF($B$2:$B$31,N13)</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.3">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
+        <v>69</v>
+      </c>
+      <c r="B14" t="s">
         <v>70</v>
       </c>
-      <c r="B14" t="s">
+      <c r="C14" t="s">
         <v>71</v>
-      </c>
-      <c r="C14" t="s">
-        <v>72</v>
       </c>
       <c r="D14" s="1">
         <v>9569270810</v>
       </c>
       <c r="E14" t="s">
+        <v>72</v>
+      </c>
+      <c r="F14" t="s">
         <v>73</v>
-      </c>
-      <c r="F14" t="s">
-        <v>74</v>
       </c>
       <c r="G14" s="3">
         <v>45901</v>
@@ -2145,7 +2138,7 @@
         <v>-6716</v>
       </c>
       <c r="I14" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="J14" t="str">
         <f t="shared" si="0"/>
@@ -2160,7 +2153,7 @@
         <v>pooja.das14@example.com</v>
       </c>
       <c r="M14">
-        <f>COUNTIF($C$2:$C$31,L14)</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="N14" t="str">
@@ -2168,28 +2161,28 @@
         <v>Pooja Das</v>
       </c>
       <c r="O14">
-        <f>COUNTIF($B$2:$B$31,N14)</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" spans="1:15" s="9" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="7" t="s">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>138</v>
+      </c>
+      <c r="B15" t="s">
+        <v>139</v>
+      </c>
+      <c r="C15" t="s">
         <v>140</v>
       </c>
-      <c r="B15" s="7" t="s">
+      <c r="D15" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="C15" s="7" t="s">
+      <c r="E15" t="s">
         <v>142</v>
       </c>
-      <c r="D15" s="1" t="s">
-        <v>143</v>
-      </c>
-      <c r="E15" s="7" t="s">
-        <v>144</v>
-      </c>
-      <c r="F15" s="7" t="s">
-        <v>26</v>
+      <c r="F15" t="s">
+        <v>25</v>
       </c>
       <c r="G15" s="3">
         <v>46012</v>
@@ -2197,52 +2190,52 @@
       <c r="H15" s="5">
         <v>17984</v>
       </c>
-      <c r="I15" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="J15" s="9" t="str">
+      <c r="I15" t="s">
+        <v>26</v>
+      </c>
+      <c r="J15" t="str">
         <f>IF(OR(M15&gt;1,O15&gt;1),"Review","OK")</f>
         <v>OK</v>
       </c>
-      <c r="K15" s="9" t="str">
+      <c r="K15" t="str">
         <f>PROPER(TRIM(customer_data[[#This Row],[City]]))</f>
         <v>Ahmedabad</v>
       </c>
-      <c r="L15" s="6" t="str">
+      <c r="L15" t="str">
         <f>TRIM(LOWER(customer_data[[#This Row],[Email]]))</f>
         <v>aditi.rao16@example.com</v>
       </c>
-      <c r="M15" s="9">
-        <f>COUNTIF($C$2:$C$31,L15)</f>
-        <v>1</v>
-      </c>
-      <c r="N15" s="9" t="str">
+      <c r="M15">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="N15" t="str">
         <f>TRIM(PROPER(customer_data[[#This Row],[Full Name]]))</f>
         <v>Aditi Rao</v>
       </c>
-      <c r="O15" s="9">
-        <f>COUNTIF($B$2:$B$31,N15)</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="O15">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>74</v>
+      </c>
+      <c r="B16" t="s">
         <v>75</v>
       </c>
-      <c r="B16" t="s">
+      <c r="C16" t="s">
         <v>76</v>
       </c>
-      <c r="C16" t="s">
+      <c r="D16" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="D16" s="1" t="s">
-        <v>78</v>
-      </c>
       <c r="E16" t="s">
+        <v>72</v>
+      </c>
+      <c r="F16" t="s">
         <v>73</v>
-      </c>
-      <c r="F16" t="s">
-        <v>74</v>
       </c>
       <c r="G16" s="3">
         <v>45725</v>
@@ -2251,7 +2244,7 @@
         <v>1862</v>
       </c>
       <c r="I16" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="J16" t="str">
         <f t="shared" si="0"/>
@@ -2266,7 +2259,7 @@
         <v>aarav.joshi17@example.com</v>
       </c>
       <c r="M16">
-        <f>COUNTIF($C$2:$C$31,L16)</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="N16" t="str">
@@ -2274,28 +2267,28 @@
         <v>Aarav Joshi</v>
       </c>
       <c r="O16">
-        <f>COUNTIF($B$2:$B$31,N16)</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.3">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
+        <v>78</v>
+      </c>
+      <c r="B17" t="s">
         <v>79</v>
       </c>
-      <c r="B17" t="s">
+      <c r="C17" t="s">
         <v>80</v>
-      </c>
-      <c r="C17" t="s">
-        <v>81</v>
       </c>
       <c r="D17" s="1">
         <v>9495084811</v>
       </c>
       <c r="E17" t="s">
+        <v>24</v>
+      </c>
+      <c r="F17" t="s">
         <v>25</v>
-      </c>
-      <c r="F17" t="s">
-        <v>26</v>
       </c>
       <c r="G17" s="3">
         <v>45561</v>
@@ -2304,7 +2297,7 @@
         <v>23804</v>
       </c>
       <c r="I17" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="J17" t="str">
         <f t="shared" si="0"/>
@@ -2319,7 +2312,7 @@
         <v>devansh.rao18@example.com</v>
       </c>
       <c r="M17">
-        <f>COUNTIF($C$2:$C$31,L17)</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="N17" t="str">
@@ -2327,28 +2320,28 @@
         <v>Devansh Rao</v>
       </c>
       <c r="O17">
-        <f>COUNTIF($B$2:$B$31,N17)</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.3">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
+        <v>81</v>
+      </c>
+      <c r="B18" t="s">
         <v>82</v>
       </c>
-      <c r="B18" t="s">
+      <c r="C18" t="s">
         <v>83</v>
       </c>
-      <c r="C18" t="s">
-        <v>84</v>
-      </c>
       <c r="D18" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="E18" t="s">
+        <v>18</v>
+      </c>
+      <c r="F18" t="s">
         <v>19</v>
-      </c>
-      <c r="F18" t="s">
-        <v>20</v>
       </c>
       <c r="G18" s="3">
         <v>45772</v>
@@ -2357,7 +2350,7 @@
         <v>17282</v>
       </c>
       <c r="I18" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="J18" t="str">
         <f t="shared" si="0"/>
@@ -2372,7 +2365,7 @@
         <v>siddharth.patel19@example.com</v>
       </c>
       <c r="M18">
-        <f>COUNTIF($C$2:$C$31,L18)</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="N18" t="str">
@@ -2380,28 +2373,28 @@
         <v>Siddharth Patel</v>
       </c>
       <c r="O18">
-        <f>COUNTIF($B$2:$B$31,N18)</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.3">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
+        <v>84</v>
+      </c>
+      <c r="B19" t="s">
         <v>85</v>
       </c>
-      <c r="B19" t="s">
+      <c r="C19" t="s">
         <v>86</v>
-      </c>
-      <c r="C19" t="s">
-        <v>87</v>
       </c>
       <c r="D19" s="1">
         <v>9137343472</v>
       </c>
       <c r="E19" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F19" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="G19" s="3">
         <v>45611</v>
@@ -2410,7 +2403,7 @@
         <v>2150</v>
       </c>
       <c r="I19" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="J19" t="str">
         <f t="shared" si="0"/>
@@ -2425,7 +2418,7 @@
         <v>arjun.verma20@example.com</v>
       </c>
       <c r="M19">
-        <f>COUNTIF($C$2:$C$31,L19)</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="N19" t="str">
@@ -2433,28 +2426,28 @@
         <v>Arjun Verma</v>
       </c>
       <c r="O19">
-        <f>COUNTIF($B$2:$B$31,N19)</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.3">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
+        <v>88</v>
+      </c>
+      <c r="B20" t="s">
         <v>89</v>
       </c>
-      <c r="B20" t="s">
+      <c r="C20" t="s">
         <v>90</v>
-      </c>
-      <c r="C20" t="s">
-        <v>91</v>
       </c>
       <c r="D20" s="1">
         <v>9403422088</v>
       </c>
       <c r="E20" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="F20" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G20" s="3">
         <v>46115</v>
@@ -2463,7 +2456,7 @@
         <v>23979</v>
       </c>
       <c r="I20" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="J20" t="str">
         <f t="shared" si="0"/>
@@ -2478,7 +2471,7 @@
         <v>aditya.menon21@example.com</v>
       </c>
       <c r="M20">
-        <f>COUNTIF($C$2:$C$31,L20)</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="N20" t="str">
@@ -2486,28 +2479,28 @@
         <v>Aditya Menon</v>
       </c>
       <c r="O20">
-        <f>COUNTIF($B$2:$B$31,N20)</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.3">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
+        <v>92</v>
+      </c>
+      <c r="B21" t="s">
         <v>93</v>
       </c>
-      <c r="B21" t="s">
+      <c r="C21" t="s">
         <v>94</v>
-      </c>
-      <c r="C21" t="s">
-        <v>95</v>
       </c>
       <c r="D21" s="1">
         <v>9256982177</v>
       </c>
       <c r="E21" t="s">
+        <v>44</v>
+      </c>
+      <c r="F21" t="s">
         <v>45</v>
-      </c>
-      <c r="F21" t="s">
-        <v>46</v>
       </c>
       <c r="G21" s="3">
         <v>45293</v>
@@ -2516,7 +2509,7 @@
         <v>15575</v>
       </c>
       <c r="I21" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="J21" t="str">
         <f t="shared" si="0"/>
@@ -2531,7 +2524,7 @@
         <v>diya.sharma22@example.com</v>
       </c>
       <c r="M21">
-        <f>COUNTIF($C$2:$C$31,L21)</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="N21" t="str">
@@ -2539,28 +2532,28 @@
         <v>Diya Sharma</v>
       </c>
       <c r="O21">
-        <f>COUNTIF($B$2:$B$31,N21)</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.3">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
+        <v>95</v>
+      </c>
+      <c r="B22" t="s">
         <v>96</v>
       </c>
-      <c r="B22" t="s">
+      <c r="C22" t="s">
         <v>97</v>
       </c>
-      <c r="C22" t="s">
+      <c r="D22" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="D22" s="1" t="s">
+      <c r="E22" t="s">
+        <v>129</v>
+      </c>
+      <c r="F22" t="s">
         <v>99</v>
-      </c>
-      <c r="E22" t="s">
-        <v>131</v>
-      </c>
-      <c r="F22" t="s">
-        <v>100</v>
       </c>
       <c r="G22" s="3">
         <v>45546</v>
@@ -2569,7 +2562,7 @@
         <v>14121</v>
       </c>
       <c r="I22" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="J22" t="str">
         <f t="shared" si="0"/>
@@ -2584,7 +2577,7 @@
         <v>simran.menon23@example.com</v>
       </c>
       <c r="M22">
-        <f>COUNTIF($C$2:$C$31,L22)</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="N22" t="str">
@@ -2592,28 +2585,28 @@
         <v>Simran Menon</v>
       </c>
       <c r="O22">
-        <f>COUNTIF($B$2:$B$31,N22)</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.3">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
+        <v>100</v>
+      </c>
+      <c r="B23" t="s">
+        <v>22</v>
+      </c>
+      <c r="C23" t="s">
+        <v>128</v>
+      </c>
+      <c r="D23" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="B23" t="s">
-        <v>23</v>
-      </c>
-      <c r="C23" t="s">
-        <v>130</v>
-      </c>
-      <c r="D23" s="1" t="s">
-        <v>102</v>
-      </c>
       <c r="E23" t="s">
+        <v>54</v>
+      </c>
+      <c r="F23" t="s">
         <v>55</v>
-      </c>
-      <c r="F23" t="s">
-        <v>56</v>
       </c>
       <c r="G23" s="3">
         <v>45324</v>
@@ -2622,7 +2615,7 @@
         <v>37273</v>
       </c>
       <c r="I23" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="J23" t="str">
         <f t="shared" si="0"/>
@@ -2637,7 +2630,7 @@
         <v>not provided</v>
       </c>
       <c r="M23">
-        <f>COUNTIF($C$2:$C$31,L23)</f>
+        <f t="shared" si="1"/>
         <v>4</v>
       </c>
       <c r="N23" t="str">
@@ -2645,28 +2638,28 @@
         <v>Ananya Bhatt</v>
       </c>
       <c r="O23">
-        <f>COUNTIF($B$2:$B$31,N23)</f>
+        <f t="shared" si="2"/>
         <v>2</v>
       </c>
     </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
+        <v>102</v>
+      </c>
+      <c r="B24" t="s">
+        <v>57</v>
+      </c>
+      <c r="C24" t="s">
         <v>103</v>
-      </c>
-      <c r="B24" t="s">
-        <v>58</v>
-      </c>
-      <c r="C24" t="s">
-        <v>104</v>
       </c>
       <c r="D24" s="1">
         <v>9311880275</v>
       </c>
       <c r="E24" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="F24" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G24" s="3">
         <v>45794</v>
@@ -2675,7 +2668,7 @@
         <v>25673</v>
       </c>
       <c r="I24" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="J24" t="str">
         <f t="shared" si="0"/>
@@ -2690,7 +2683,7 @@
         <v>siddharth.kapoor25@example.com</v>
       </c>
       <c r="M24">
-        <f>COUNTIF($C$2:$C$31,L24)</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="N24" t="str">
@@ -2698,28 +2691,28 @@
         <v>Siddharth Kapoor</v>
       </c>
       <c r="O24">
-        <f>COUNTIF($B$2:$B$31,N24)</f>
+        <f t="shared" si="2"/>
         <v>2</v>
       </c>
     </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
+        <v>104</v>
+      </c>
+      <c r="B25" t="s">
         <v>105</v>
       </c>
-      <c r="B25" t="s">
+      <c r="C25" t="s">
         <v>106</v>
       </c>
-      <c r="C25" t="s">
+      <c r="D25" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="E25" t="s">
         <v>107</v>
       </c>
-      <c r="D25" s="1" t="s">
-        <v>130</v>
-      </c>
-      <c r="E25" t="s">
-        <v>108</v>
-      </c>
       <c r="F25" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G25" s="3">
         <v>45791</v>
@@ -2728,7 +2721,7 @@
         <v>40656</v>
       </c>
       <c r="I25" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="J25" t="str">
         <f t="shared" si="0"/>
@@ -2743,7 +2736,7 @@
         <v>arjun.menon26@example.com</v>
       </c>
       <c r="M25">
-        <f>COUNTIF($C$2:$C$31,L25)</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="N25" t="str">
@@ -2751,28 +2744,28 @@
         <v>Arjun Menon</v>
       </c>
       <c r="O25">
-        <f>COUNTIF($B$2:$B$31,N25)</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.3">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
+        <v>108</v>
+      </c>
+      <c r="B26" t="s">
         <v>109</v>
       </c>
-      <c r="B26" t="s">
+      <c r="C26" t="s">
         <v>110</v>
-      </c>
-      <c r="C26" t="s">
-        <v>111</v>
       </c>
       <c r="D26" s="1">
         <v>9561072854</v>
       </c>
       <c r="E26" t="s">
+        <v>24</v>
+      </c>
+      <c r="F26" t="s">
         <v>25</v>
-      </c>
-      <c r="F26" t="s">
-        <v>26</v>
       </c>
       <c r="G26" s="3">
         <v>46084</v>
@@ -2781,7 +2774,7 @@
         <v>22745</v>
       </c>
       <c r="I26" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="J26" t="str">
         <f t="shared" si="0"/>
@@ -2796,7 +2789,7 @@
         <v>rohan.kapoor27@example.com</v>
       </c>
       <c r="M26">
-        <f>COUNTIF($C$2:$C$31,L26)</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="N26" t="str">
@@ -2804,28 +2797,28 @@
         <v>Rohan Kapoor</v>
       </c>
       <c r="O26">
-        <f>COUNTIF($B$2:$B$31,N26)</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.3">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
+        <v>111</v>
+      </c>
+      <c r="B27" t="s">
         <v>112</v>
       </c>
-      <c r="B27" t="s">
+      <c r="C27" t="s">
         <v>113</v>
       </c>
-      <c r="C27" t="s">
+      <c r="D27" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="D27" s="1" t="s">
-        <v>115</v>
-      </c>
       <c r="E27" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="F27" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G27" s="3">
         <v>45497</v>
@@ -2834,7 +2827,7 @@
         <v>4075</v>
       </c>
       <c r="I27" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="J27" t="str">
         <f t="shared" si="0"/>
@@ -2849,7 +2842,7 @@
         <v>sneha.chauhan28@example.com</v>
       </c>
       <c r="M27">
-        <f>COUNTIF($C$2:$C$31,L27)</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="N27" t="str">
@@ -2857,28 +2850,28 @@
         <v>Sneha Chauhan</v>
       </c>
       <c r="O27">
-        <f>COUNTIF($B$2:$B$31,N27)</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.3">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
+        <v>115</v>
+      </c>
+      <c r="B28" t="s">
         <v>116</v>
       </c>
-      <c r="B28" t="s">
+      <c r="C28" t="s">
         <v>117</v>
       </c>
-      <c r="C28" t="s">
+      <c r="D28" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="D28" s="1" t="s">
-        <v>119</v>
-      </c>
       <c r="E28" t="s">
+        <v>24</v>
+      </c>
+      <c r="F28" t="s">
         <v>25</v>
-      </c>
-      <c r="F28" t="s">
-        <v>26</v>
       </c>
       <c r="G28" s="3">
         <v>45420</v>
@@ -2887,7 +2880,7 @@
         <v>36196</v>
       </c>
       <c r="I28" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="J28" t="str">
         <f t="shared" si="0"/>
@@ -2902,7 +2895,7 @@
         <v>meera.reddy29@example.com</v>
       </c>
       <c r="M28">
-        <f>COUNTIF($C$2:$C$31,L28)</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="N28" t="str">
@@ -2910,28 +2903,28 @@
         <v>Meera Reddy</v>
       </c>
       <c r="O28">
-        <f>COUNTIF($B$2:$B$31,N28)</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.3">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
+        <v>119</v>
+      </c>
+      <c r="B29" t="s">
         <v>120</v>
       </c>
-      <c r="B29" t="s">
-        <v>121</v>
-      </c>
       <c r="C29" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="D29" s="1">
         <v>9214210239</v>
       </c>
       <c r="E29" t="s">
+        <v>31</v>
+      </c>
+      <c r="F29" t="s">
         <v>32</v>
-      </c>
-      <c r="F29" t="s">
-        <v>33</v>
       </c>
       <c r="G29" s="3">
         <v>46012</v>
@@ -2940,7 +2933,7 @@
         <v>24656</v>
       </c>
       <c r="I29" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="J29" t="str">
         <f t="shared" si="0"/>
@@ -2955,7 +2948,7 @@
         <v>not provided</v>
       </c>
       <c r="M29">
-        <f>COUNTIF($C$2:$C$31,L29)</f>
+        <f t="shared" si="1"/>
         <v>4</v>
       </c>
       <c r="N29" t="str">
@@ -2963,28 +2956,28 @@
         <v>Vivaan Chauhan</v>
       </c>
       <c r="O29">
-        <f>COUNTIF($B$2:$B$31,N29)</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.3">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
+        <v>121</v>
+      </c>
+      <c r="B30" t="s">
+        <v>143</v>
+      </c>
+      <c r="C30" t="s">
         <v>122</v>
-      </c>
-      <c r="B30" t="s">
-        <v>123</v>
-      </c>
-      <c r="C30" t="s">
-        <v>124</v>
       </c>
       <c r="D30" s="1">
         <v>9222271940</v>
       </c>
       <c r="E30" t="s">
+        <v>18</v>
+      </c>
+      <c r="F30" t="s">
         <v>19</v>
-      </c>
-      <c r="F30" t="s">
-        <v>20</v>
       </c>
       <c r="G30" s="3">
         <v>45892</v>
@@ -2993,7 +2986,7 @@
         <v>6593</v>
       </c>
       <c r="I30" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="J30" t="str">
         <f t="shared" si="0"/>
@@ -3008,7 +3001,7 @@
         <v>anika.gupta12@example.com</v>
       </c>
       <c r="M30">
-        <f>COUNTIF($C$2:$C$31,L30)</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="N30" t="str">
@@ -3016,28 +3009,28 @@
         <v>Anika Gupta</v>
       </c>
       <c r="O30">
-        <f>COUNTIF($B$2:$B$31,N30)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.3">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
+        <v>123</v>
+      </c>
+      <c r="B31" t="s">
+        <v>124</v>
+      </c>
+      <c r="C31" t="s">
         <v>125</v>
-      </c>
-      <c r="B31" t="s">
-        <v>126</v>
-      </c>
-      <c r="C31" t="s">
-        <v>127</v>
       </c>
       <c r="D31" s="1">
         <v>9353685732</v>
       </c>
       <c r="E31" t="s">
+        <v>24</v>
+      </c>
+      <c r="F31" t="s">
         <v>25</v>
-      </c>
-      <c r="F31" t="s">
-        <v>26</v>
       </c>
       <c r="G31" s="3">
         <v>46178</v>
@@ -3046,7 +3039,7 @@
         <v>-40828</v>
       </c>
       <c r="I31" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="J31" t="str">
         <f t="shared" si="0"/>
@@ -3061,7 +3054,7 @@
         <v>pooja.gupta15@example.com</v>
       </c>
       <c r="M31">
-        <f>COUNTIF($C$2:$C$31,L31)</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="N31" t="str">
@@ -3069,21 +3062,21 @@
         <v>Pooja Gupta</v>
       </c>
       <c r="O31">
-        <f>COUNTIF($B$2:$B$31,N31)</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C35" s="2">
         <f>COUNTBLANK(customer_data[Email])</f>
         <v>0</v>
@@ -3108,76 +3101,76 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{58D3BD0D-8D3C-4D7D-8184-B43C65FDEBB3}">
   <dimension ref="A1:B8"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.21875" customWidth="1"/>
+    <col min="1" max="1" width="24.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="B1">
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A2" s="8" t="s">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>131</v>
+      </c>
+      <c r="B2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>132</v>
+      </c>
+      <c r="B3">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>133</v>
       </c>
-      <c r="B2" s="8">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A3" s="8" t="s">
-        <v>134</v>
-      </c>
-      <c r="B3" s="8">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A4" s="8" t="s">
-        <v>135</v>
-      </c>
-      <c r="B4" s="9">
+      <c r="B4">
         <f>COUNTA(customer_data[Customer ID])</f>
         <v>30</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A5" s="8" t="s">
-        <v>136</v>
-      </c>
-      <c r="B5" s="8">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>134</v>
+      </c>
+      <c r="B5">
         <f>COUNTIF(customer_data[Email],"Not Provided")</f>
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A6" s="8" t="s">
-        <v>139</v>
-      </c>
-      <c r="B6" s="8">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>137</v>
+      </c>
+      <c r="B6">
         <f>COUNTIF(customer_data[Phone],"Not Provided")</f>
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A7" s="8" t="s">
-        <v>137</v>
-      </c>
-      <c r="B7" s="8">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>135</v>
+      </c>
+      <c r="B7">
         <f>COUNTIF(customer_data[City],"Unknown")</f>
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A8" s="8" t="s">
-        <v>138</v>
-      </c>
-      <c r="B8" s="8">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>136</v>
+      </c>
+      <c r="B8">
         <f>COUNTIF(customer_data[Total Purchases],"&lt;0")</f>
         <v>2</v>
       </c>

</xml_diff>